<commit_message>
dados: 2026-10-14 08:21 (132 arquivos)
</commit_message>
<xml_diff>
--- a/xlsx/dre/DRE_02_2026.xlsx
+++ b/xlsx/dre/DRE_02_2026.xlsx
@@ -1550,6 +1550,12 @@
     <t>R$ 10.123,95</t>
   </si>
   <si>
+    <t>R$  1.108,54</t>
+  </si>
+  <si>
+    <t>R$  1.196,02</t>
+  </si>
+  <si>
     <t>RAYSSA BARBOSA SILVA</t>
   </si>
   <si>
@@ -1562,31 +1568,25 @@
     <t>FERNANDA DOCHVAT SILVA</t>
   </si>
   <si>
+    <t>01/06/26</t>
+  </si>
+  <si>
     <t>01/04/26</t>
   </si>
   <si>
-    <t>R$  1.196,02</t>
-  </si>
-  <si>
-    <t>01/06/26</t>
-  </si>
-  <si>
-    <t>R$  1.108,54</t>
+    <t>R$  438,09</t>
+  </si>
+  <si>
+    <t>R$  3,60</t>
   </si>
   <si>
     <t>63801/2</t>
   </si>
   <si>
-    <t>R$  438,09</t>
+    <t>R$  537,59</t>
   </si>
   <si>
     <t>R$  292,95</t>
-  </si>
-  <si>
-    <t>R$  537,59</t>
-  </si>
-  <si>
-    <t>R$  3,60</t>
   </si>
   <si>
     <t>R$  1.941,34</t>
@@ -2028,15 +2028,15 @@
     <t>4.03.03.02.05.02 Assistência técnica medição</t>
   </si>
   <si>
+    <t>PFP</t>
+  </si>
+  <si>
     <t>L E A Medicoes Tecnicas LTDA</t>
   </si>
   <si>
     <t>R$  180,00</t>
   </si>
   <si>
-    <t>PFP</t>
-  </si>
-  <si>
     <t>4.03.03.09 Marketing - mídias / ações comerciais / outros (CV)</t>
   </si>
   <si>
@@ -2058,6 +2058,18 @@
     <t>Google 2026</t>
   </si>
   <si>
+    <t>498/1</t>
+  </si>
+  <si>
+    <t>Facebook</t>
+  </si>
+  <si>
+    <t>R$  3.750,00</t>
+  </si>
+  <si>
+    <t>30/01/26</t>
+  </si>
+  <si>
     <t>WEBGIGA SOLUCOES DIGITAIS LTDA</t>
   </si>
   <si>
@@ -2079,18 +2091,6 @@
     <t>MHM - Honorários 2026</t>
   </si>
   <si>
-    <t>498/1</t>
-  </si>
-  <si>
-    <t>Facebook</t>
-  </si>
-  <si>
-    <t>R$  3.750,00</t>
-  </si>
-  <si>
-    <t>30/01/26</t>
-  </si>
-  <si>
     <t>4.04 DESPESAS ADMINISTRATIVAS</t>
   </si>
   <si>
@@ -2136,40 +2136,70 @@
     <t>4.04.01.02.01.01 Salário fixo</t>
   </si>
   <si>
+    <t>Bianca Rodrigues - Salário fixo 2026</t>
+  </si>
+  <si>
+    <t>587/1</t>
+  </si>
+  <si>
+    <t>R$  2.075,32</t>
+  </si>
+  <si>
+    <t>Rateio salários Mayara, Rayssa e Efraim</t>
+  </si>
+  <si>
+    <t>Fernanda Dochvat - Fixo 2026</t>
+  </si>
+  <si>
+    <t>Danielle Martins da Silva</t>
+  </si>
+  <si>
+    <t>R$  2.090,00</t>
+  </si>
+  <si>
+    <t>Danielle - Pagamento 2026</t>
+  </si>
+  <si>
+    <t>GUTEMBERG DIAS GOMES</t>
+  </si>
+  <si>
+    <t>R$  6.000,00</t>
+  </si>
+  <si>
+    <t>Gutemberg Dias - Pagamento</t>
+  </si>
+  <si>
+    <t>Leandro Henrique Simoes Campos</t>
+  </si>
+  <si>
+    <t>R$  2.000,00</t>
+  </si>
+  <si>
+    <t>Leandro Henrique Simoes Campos Fixo 2026</t>
+  </si>
+  <si>
+    <t>Carina - Pagamento 2026</t>
+  </si>
+  <si>
+    <t>Denny Lucas do Carmo Pereira</t>
+  </si>
+  <si>
+    <t>R$  2.645,58</t>
+  </si>
+  <si>
+    <t>Denny Lucas - Pagamento 2026</t>
+  </si>
+  <si>
     <t>Rubens - Pagamento 2026</t>
   </si>
   <si>
     <t>579/1</t>
   </si>
   <si>
-    <t>587/1</t>
-  </si>
-  <si>
-    <t>R$  2.075,32</t>
-  </si>
-  <si>
-    <t>Rateio salários Mayara, Rayssa e Efraim</t>
-  </si>
-  <si>
-    <t>Fernanda Dochvat - Fixo 2026</t>
-  </si>
-  <si>
-    <t>GUTEMBERG DIAS GOMES</t>
-  </si>
-  <si>
-    <t>R$  6.000,00</t>
-  </si>
-  <si>
-    <t>Gutemberg Dias - Pagamento</t>
-  </si>
-  <si>
-    <t>Denny Lucas do Carmo Pereira</t>
-  </si>
-  <si>
-    <t>R$  2.645,58</t>
-  </si>
-  <si>
-    <t>Denny Lucas - Pagamento 2026</t>
+    <t>Eric Kevin de Souza Serpa</t>
+  </si>
+  <si>
+    <t>Salário Fixo -Eric Serpa 2026</t>
   </si>
   <si>
     <t>Teresinha Elvira Maximino de Menezes</t>
@@ -2178,6 +2208,12 @@
     <t>Tucha - Fixo 2026</t>
   </si>
   <si>
+    <t>578/1</t>
+  </si>
+  <si>
+    <t>R$  2.219,85</t>
+  </si>
+  <si>
     <t>SABRINA ALVES DE ABREU BRAUNBECK</t>
   </si>
   <si>
@@ -2187,42 +2223,6 @@
     <t>Sabrina Braunbeck - Pagamento 2026</t>
   </si>
   <si>
-    <t>Leandro Henrique Simoes Campos</t>
-  </si>
-  <si>
-    <t>R$  2.000,00</t>
-  </si>
-  <si>
-    <t>Leandro Henrique Simoes Campos Fixo 2026</t>
-  </si>
-  <si>
-    <t>R$  2.090,00</t>
-  </si>
-  <si>
-    <t>Carina - Pagamento 2026</t>
-  </si>
-  <si>
-    <t>Eric Kevin de Souza Serpa</t>
-  </si>
-  <si>
-    <t>Salário Fixo -Eric Serpa 2026</t>
-  </si>
-  <si>
-    <t>Bianca Rodrigues - Salário fixo 2026</t>
-  </si>
-  <si>
-    <t>578/1</t>
-  </si>
-  <si>
-    <t>R$  2.219,85</t>
-  </si>
-  <si>
-    <t>Danielle Martins da Silva</t>
-  </si>
-  <si>
-    <t>Danielle - Pagamento 2026</t>
-  </si>
-  <si>
     <t>4.04.01.02.05 IRRF sobre salários</t>
   </si>
   <si>
@@ -2292,12 +2292,12 @@
     <t>VT fev 26/1</t>
   </si>
   <si>
+    <t>R$  433,98</t>
+  </si>
+  <si>
     <t>R$  313,70</t>
   </si>
   <si>
-    <t>R$  433,98</t>
-  </si>
-  <si>
     <t>4.04.02 GASTOS GERAIS ADMINISTRATIVOS</t>
   </si>
   <si>
@@ -2436,17 +2436,25 @@
     <t>R$  45,00</t>
   </si>
   <si>
-    <t>531/1</t>
-  </si>
-  <si>
-    <t>Shopee</t>
-  </si>
-  <si>
-    <t>R$  65,93</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Freeco refil
-</t>
+    <t>532/1</t>
+  </si>
+  <si>
+    <t>DIA BRASIL SUPERMERCADO</t>
+  </si>
+  <si>
+    <t>R$  59,96</t>
+  </si>
+  <si>
+    <t>cafés</t>
+  </si>
+  <si>
+    <t>502/1</t>
+  </si>
+  <si>
+    <t>R$  100,00</t>
+  </si>
+  <si>
+    <t>Cópia de chaves</t>
   </si>
   <si>
     <t>533/1</t>
@@ -2459,19 +2467,6 @@
   </si>
   <si>
     <t>material limpeza</t>
-  </si>
-  <si>
-    <t>530/1</t>
-  </si>
-  <si>
-    <t>Marinete</t>
-  </si>
-  <si>
-    <t>R$  17,00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Copo descartável para crianças
-</t>
   </si>
   <si>
     <t>529/1</t>
@@ -2488,27 +2483,6 @@
 </t>
   </si>
   <si>
-    <t>502/1</t>
-  </si>
-  <si>
-    <t>R$  100,00</t>
-  </si>
-  <si>
-    <t>Cópia de chaves</t>
-  </si>
-  <si>
-    <t>532/1</t>
-  </si>
-  <si>
-    <t>DIA BRASIL SUPERMERCADO</t>
-  </si>
-  <si>
-    <t>R$  59,96</t>
-  </si>
-  <si>
-    <t>cafés</t>
-  </si>
-  <si>
     <t>505/1</t>
   </si>
   <si>
@@ -2521,6 +2495,32 @@
     <t>Conserto vidro adega</t>
   </si>
   <si>
+    <t>531/1</t>
+  </si>
+  <si>
+    <t>Shopee</t>
+  </si>
+  <si>
+    <t>R$  65,93</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Freeco refil
+</t>
+  </si>
+  <si>
+    <t>530/1</t>
+  </si>
+  <si>
+    <t>Marinete</t>
+  </si>
+  <si>
+    <t>R$  17,00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Copo descartável para crianças
+</t>
+  </si>
+  <si>
     <t>4.04.02.07 Informática</t>
   </si>
   <si>
@@ -2584,6 +2584,15 @@
     <t>4.04.02.08.03 Mensalidades e assinaturas - outros gastos</t>
   </si>
   <si>
+    <t>D4 sign</t>
+  </si>
+  <si>
+    <t>R$  49,95</t>
+  </si>
+  <si>
+    <t>D4 sign 2026</t>
+  </si>
+  <si>
     <t>534/1</t>
   </si>
   <si>
@@ -2593,15 +2602,6 @@
     <t>R$  197,63</t>
   </si>
   <si>
-    <t>D4 sign</t>
-  </si>
-  <si>
-    <t>R$  49,95</t>
-  </si>
-  <si>
-    <t>D4 sign 2026</t>
-  </si>
-  <si>
     <t>10/2</t>
   </si>
   <si>
@@ -2614,6 +2614,12 @@
     <t>Promob 2026-1</t>
   </si>
   <si>
+    <t>R$  599,00</t>
+  </si>
+  <si>
+    <t>Promob 2026</t>
+  </si>
+  <si>
     <t>3/1</t>
   </si>
   <si>
@@ -2621,12 +2627,6 @@
   </si>
   <si>
     <t>Promob 2026/2</t>
-  </si>
-  <si>
-    <t>R$  599,00</t>
-  </si>
-  <si>
-    <t>Promob 2026</t>
   </si>
   <si>
     <t>4.04.02.11 Manutenção de predio e equipamentos</t>
@@ -2723,6 +2723,15 @@
     <t>R$ 400,33</t>
   </si>
   <si>
+    <t>VERISURE</t>
+  </si>
+  <si>
+    <t>R$  250,33</t>
+  </si>
+  <si>
+    <t>Verisure - Alarme 2026</t>
+  </si>
+  <si>
     <t>Jackson Fernando de Araujo</t>
   </si>
   <si>
@@ -2730,15 +2739,6 @@
   </si>
   <si>
     <t>Segurança 2026</t>
-  </si>
-  <si>
-    <t>VERISURE</t>
-  </si>
-  <si>
-    <t>R$  250,33</t>
-  </si>
-  <si>
-    <t>Verisure - Alarme 2026</t>
   </si>
   <si>
     <t>4.04.02.14.08 Site e newsletter da loja</t>
@@ -15554,7 +15554,7 @@
         <v>33</v>
       </c>
       <c r="E234" t="s">
-        <v>244</v>
+        <v>275</v>
       </c>
       <c r="F234" t="s">
         <v>218</v>
@@ -15563,16 +15563,16 @@
         <v>41</v>
       </c>
       <c r="H234" t="s">
+        <v>457</v>
+      </c>
+      <c r="I234" t="s">
         <v>508</v>
       </c>
-      <c r="I234" t="s">
-        <v>509</v>
-      </c>
       <c r="J234" t="s">
-        <v>510</v>
+        <v>304</v>
       </c>
       <c r="K234" t="s">
-        <v>80</v>
+        <v>58</v>
       </c>
       <c r="L234" t="s">
         <v>34</v>
@@ -15584,10 +15584,10 @@
         <v>47</v>
       </c>
       <c r="O234" t="s">
-        <v>247</v>
+        <v>105</v>
       </c>
       <c r="P234" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="Q234" t="s">
         <v>47</v>
@@ -15610,7 +15610,7 @@
         <v>34</v>
       </c>
       <c r="E235" t="s">
-        <v>251</v>
+        <v>234</v>
       </c>
       <c r="F235" t="s">
         <v>218</v>
@@ -15619,16 +15619,16 @@
         <v>41</v>
       </c>
       <c r="H235" t="s">
-        <v>511</v>
+        <v>457</v>
       </c>
       <c r="I235" t="s">
-        <v>430</v>
+        <v>509</v>
       </c>
       <c r="J235" t="s">
-        <v>512</v>
+        <v>300</v>
       </c>
       <c r="K235" t="s">
-        <v>70</v>
+        <v>119</v>
       </c>
       <c r="L235" t="s">
         <v>34</v>
@@ -15640,10 +15640,10 @@
         <v>47</v>
       </c>
       <c r="O235" t="s">
-        <v>71</v>
+        <v>130</v>
       </c>
       <c r="P235" t="s">
-        <v>430</v>
+        <v>509</v>
       </c>
       <c r="Q235" t="s">
         <v>47</v>
@@ -15666,7 +15666,7 @@
         <v>34</v>
       </c>
       <c r="E236" t="s">
-        <v>223</v>
+        <v>244</v>
       </c>
       <c r="F236" t="s">
         <v>218</v>
@@ -15675,16 +15675,16 @@
         <v>41</v>
       </c>
       <c r="H236" t="s">
+        <v>510</v>
+      </c>
+      <c r="I236" t="s">
         <v>511</v>
-      </c>
-      <c r="I236" t="s">
-        <v>439</v>
       </c>
       <c r="J236" t="s">
         <v>512</v>
       </c>
       <c r="K236" t="s">
-        <v>113</v>
+        <v>80</v>
       </c>
       <c r="L236" t="s">
         <v>34</v>
@@ -15696,10 +15696,10 @@
         <v>47</v>
       </c>
       <c r="O236" t="s">
-        <v>114</v>
+        <v>247</v>
       </c>
       <c r="P236" t="s">
-        <v>439</v>
+        <v>511</v>
       </c>
       <c r="Q236" t="s">
         <v>47</v>
@@ -15722,7 +15722,7 @@
         <v>34</v>
       </c>
       <c r="E237" t="s">
-        <v>234</v>
+        <v>248</v>
       </c>
       <c r="F237" t="s">
         <v>218</v>
@@ -15731,10 +15731,10 @@
         <v>41</v>
       </c>
       <c r="H237" t="s">
-        <v>457</v>
+        <v>513</v>
       </c>
       <c r="I237" t="s">
-        <v>513</v>
+        <v>428</v>
       </c>
       <c r="J237" t="s">
         <v>300</v>
@@ -15752,10 +15752,10 @@
         <v>47</v>
       </c>
       <c r="O237" t="s">
-        <v>130</v>
+        <v>250</v>
       </c>
       <c r="P237" t="s">
-        <v>513</v>
+        <v>428</v>
       </c>
       <c r="Q237" t="s">
         <v>47</v>
@@ -15778,7 +15778,7 @@
         <v>34</v>
       </c>
       <c r="E238" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="F238" t="s">
         <v>218</v>
@@ -15787,16 +15787,16 @@
         <v>41</v>
       </c>
       <c r="H238" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="I238" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="J238" t="s">
-        <v>300</v>
+        <v>514</v>
       </c>
       <c r="K238" t="s">
-        <v>119</v>
+        <v>80</v>
       </c>
       <c r="L238" t="s">
         <v>34</v>
@@ -15808,10 +15808,10 @@
         <v>47</v>
       </c>
       <c r="O238" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="P238" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="Q238" t="s">
         <v>47</v>
@@ -15834,7 +15834,7 @@
         <v>34</v>
       </c>
       <c r="E239" t="s">
-        <v>253</v>
+        <v>223</v>
       </c>
       <c r="F239" t="s">
         <v>218</v>
@@ -15843,16 +15843,16 @@
         <v>41</v>
       </c>
       <c r="H239" t="s">
-        <v>508</v>
+        <v>513</v>
       </c>
       <c r="I239" t="s">
-        <v>429</v>
+        <v>439</v>
       </c>
       <c r="J239" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="K239" t="s">
-        <v>80</v>
+        <v>113</v>
       </c>
       <c r="L239" t="s">
         <v>34</v>
@@ -15864,10 +15864,10 @@
         <v>47</v>
       </c>
       <c r="O239" t="s">
-        <v>255</v>
+        <v>114</v>
       </c>
       <c r="P239" t="s">
-        <v>429</v>
+        <v>439</v>
       </c>
       <c r="Q239" t="s">
         <v>47</v>
@@ -15890,25 +15890,25 @@
         <v>34</v>
       </c>
       <c r="E240" t="s">
-        <v>232</v>
+        <v>242</v>
       </c>
       <c r="F240" t="s">
-        <v>218</v>
+        <v>499</v>
       </c>
       <c r="G240" t="s">
         <v>41</v>
       </c>
       <c r="H240" t="s">
-        <v>511</v>
+        <v>457</v>
       </c>
       <c r="I240" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="J240" t="s">
-        <v>512</v>
+        <v>80</v>
       </c>
       <c r="K240" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="L240" t="s">
         <v>34</v>
@@ -15920,13 +15920,13 @@
         <v>47</v>
       </c>
       <c r="O240" t="s">
-        <v>310</v>
+        <v>34</v>
       </c>
       <c r="P240" t="s">
-        <v>438</v>
+        <v>34</v>
       </c>
       <c r="Q240" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="R240" t="s">
         <v>34</v>
@@ -15946,25 +15946,25 @@
         <v>34</v>
       </c>
       <c r="E241" t="s">
-        <v>275</v>
+        <v>360</v>
       </c>
       <c r="F241" t="s">
-        <v>218</v>
+        <v>499</v>
       </c>
       <c r="G241" t="s">
         <v>41</v>
       </c>
       <c r="H241" t="s">
-        <v>457</v>
+        <v>215</v>
       </c>
       <c r="I241" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="J241" t="s">
-        <v>304</v>
+        <v>119</v>
       </c>
       <c r="K241" t="s">
-        <v>58</v>
+        <v>119</v>
       </c>
       <c r="L241" t="s">
         <v>34</v>
@@ -15976,13 +15976,13 @@
         <v>47</v>
       </c>
       <c r="O241" t="s">
-        <v>105</v>
+        <v>34</v>
       </c>
       <c r="P241" t="s">
-        <v>515</v>
+        <v>34</v>
       </c>
       <c r="Q241" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="R241" t="s">
         <v>34</v>
@@ -16002,25 +16002,25 @@
         <v>34</v>
       </c>
       <c r="E242" t="s">
-        <v>472</v>
+        <v>357</v>
       </c>
       <c r="F242" t="s">
-        <v>218</v>
+        <v>499</v>
       </c>
       <c r="G242" t="s">
         <v>41</v>
       </c>
       <c r="H242" t="s">
-        <v>457</v>
+        <v>215</v>
       </c>
       <c r="I242" t="s">
-        <v>473</v>
+        <v>517</v>
       </c>
       <c r="J242" t="s">
-        <v>461</v>
+        <v>80</v>
       </c>
       <c r="K242" t="s">
-        <v>113</v>
+        <v>80</v>
       </c>
       <c r="L242" t="s">
         <v>34</v>
@@ -16032,13 +16032,13 @@
         <v>47</v>
       </c>
       <c r="O242" t="s">
-        <v>475</v>
+        <v>34</v>
       </c>
       <c r="P242" t="s">
-        <v>473</v>
+        <v>34</v>
       </c>
       <c r="Q242" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="R242" t="s">
         <v>34</v>
@@ -16058,25 +16058,25 @@
         <v>34</v>
       </c>
       <c r="E243" t="s">
-        <v>516</v>
+        <v>251</v>
       </c>
       <c r="F243" t="s">
-        <v>499</v>
+        <v>218</v>
       </c>
       <c r="G243" t="s">
         <v>41</v>
       </c>
       <c r="H243" t="s">
-        <v>215</v>
+        <v>513</v>
       </c>
       <c r="I243" t="s">
-        <v>464</v>
+        <v>430</v>
       </c>
       <c r="J243" t="s">
-        <v>134</v>
+        <v>515</v>
       </c>
       <c r="K243" t="s">
-        <v>134</v>
+        <v>70</v>
       </c>
       <c r="L243" t="s">
         <v>34</v>
@@ -16088,13 +16088,13 @@
         <v>47</v>
       </c>
       <c r="O243" t="s">
-        <v>34</v>
+        <v>71</v>
       </c>
       <c r="P243" t="s">
-        <v>34</v>
+        <v>430</v>
       </c>
       <c r="Q243" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="R243" t="s">
         <v>34</v>
@@ -16114,25 +16114,25 @@
         <v>34</v>
       </c>
       <c r="E244" t="s">
-        <v>360</v>
+        <v>472</v>
       </c>
       <c r="F244" t="s">
-        <v>499</v>
+        <v>218</v>
       </c>
       <c r="G244" t="s">
         <v>41</v>
       </c>
       <c r="H244" t="s">
-        <v>215</v>
+        <v>457</v>
       </c>
       <c r="I244" t="s">
-        <v>517</v>
+        <v>473</v>
       </c>
       <c r="J244" t="s">
-        <v>119</v>
+        <v>461</v>
       </c>
       <c r="K244" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="L244" t="s">
         <v>34</v>
@@ -16144,13 +16144,13 @@
         <v>47</v>
       </c>
       <c r="O244" t="s">
-        <v>34</v>
+        <v>475</v>
       </c>
       <c r="P244" t="s">
-        <v>34</v>
+        <v>473</v>
       </c>
       <c r="Q244" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="R244" t="s">
         <v>34</v>
@@ -16170,25 +16170,25 @@
         <v>34</v>
       </c>
       <c r="E245" t="s">
-        <v>225</v>
+        <v>518</v>
       </c>
       <c r="F245" t="s">
-        <v>218</v>
+        <v>499</v>
       </c>
       <c r="G245" t="s">
         <v>41</v>
       </c>
       <c r="H245" t="s">
-        <v>457</v>
+        <v>215</v>
       </c>
       <c r="I245" t="s">
-        <v>518</v>
+        <v>464</v>
       </c>
       <c r="J245" t="s">
-        <v>304</v>
+        <v>134</v>
       </c>
       <c r="K245" t="s">
-        <v>101</v>
+        <v>134</v>
       </c>
       <c r="L245" t="s">
         <v>34</v>
@@ -16200,13 +16200,13 @@
         <v>47</v>
       </c>
       <c r="O245" t="s">
-        <v>102</v>
+        <v>34</v>
       </c>
       <c r="P245" t="s">
-        <v>518</v>
+        <v>34</v>
       </c>
       <c r="Q245" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="R245" t="s">
         <v>34</v>
@@ -16226,25 +16226,25 @@
         <v>34</v>
       </c>
       <c r="E246" t="s">
-        <v>354</v>
+        <v>232</v>
       </c>
       <c r="F246" t="s">
-        <v>499</v>
+        <v>218</v>
       </c>
       <c r="G246" t="s">
         <v>41</v>
       </c>
       <c r="H246" t="s">
-        <v>215</v>
+        <v>513</v>
       </c>
       <c r="I246" t="s">
-        <v>519</v>
+        <v>438</v>
       </c>
       <c r="J246" t="s">
+        <v>515</v>
+      </c>
+      <c r="K246" t="s">
         <v>90</v>
-      </c>
-      <c r="K246" t="s">
-        <v>229</v>
       </c>
       <c r="L246" t="s">
         <v>34</v>
@@ -16256,13 +16256,13 @@
         <v>47</v>
       </c>
       <c r="O246" t="s">
-        <v>34</v>
+        <v>310</v>
       </c>
       <c r="P246" t="s">
-        <v>34</v>
+        <v>438</v>
       </c>
       <c r="Q246" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="R246" t="s">
         <v>34</v>
@@ -16282,7 +16282,7 @@
         <v>34</v>
       </c>
       <c r="E247" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="F247" t="s">
         <v>499</v>
@@ -16294,13 +16294,13 @@
         <v>215</v>
       </c>
       <c r="I247" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="J247" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="K247" t="s">
-        <v>80</v>
+        <v>229</v>
       </c>
       <c r="L247" t="s">
         <v>34</v>
@@ -16338,25 +16338,25 @@
         <v>34</v>
       </c>
       <c r="E248" t="s">
-        <v>363</v>
+        <v>225</v>
       </c>
       <c r="F248" t="s">
-        <v>499</v>
+        <v>218</v>
       </c>
       <c r="G248" t="s">
         <v>41</v>
       </c>
       <c r="H248" t="s">
-        <v>215</v>
+        <v>457</v>
       </c>
       <c r="I248" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="J248" t="s">
-        <v>126</v>
+        <v>304</v>
       </c>
       <c r="K248" t="s">
-        <v>126</v>
+        <v>101</v>
       </c>
       <c r="L248" t="s">
         <v>34</v>
@@ -16368,13 +16368,13 @@
         <v>47</v>
       </c>
       <c r="O248" t="s">
-        <v>34</v>
+        <v>102</v>
       </c>
       <c r="P248" t="s">
-        <v>34</v>
+        <v>520</v>
       </c>
       <c r="Q248" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="R248" t="s">
         <v>34</v>
@@ -16394,7 +16394,7 @@
         <v>34</v>
       </c>
       <c r="E249" t="s">
-        <v>242</v>
+        <v>348</v>
       </c>
       <c r="F249" t="s">
         <v>499</v>
@@ -16403,16 +16403,16 @@
         <v>41</v>
       </c>
       <c r="H249" t="s">
-        <v>457</v>
+        <v>215</v>
       </c>
       <c r="I249" t="s">
-        <v>441</v>
+        <v>521</v>
       </c>
       <c r="J249" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="K249" t="s">
-        <v>80</v>
+        <v>126</v>
       </c>
       <c r="L249" t="s">
         <v>34</v>
@@ -16450,7 +16450,7 @@
         <v>34</v>
       </c>
       <c r="E250" t="s">
-        <v>348</v>
+        <v>363</v>
       </c>
       <c r="F250" t="s">
         <v>499</v>
@@ -17411,7 +17411,7 @@
         <v>41</v>
       </c>
       <c r="H267" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="I267" t="s">
         <v>554</v>
@@ -20090,25 +20090,25 @@
         <v>33</v>
       </c>
       <c r="E315" t="s">
-        <v>232</v>
+        <v>217</v>
       </c>
       <c r="F315" t="s">
-        <v>40</v>
+        <v>666</v>
       </c>
       <c r="G315" t="s">
         <v>41</v>
       </c>
       <c r="H315" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="I315" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="J315" t="s">
-        <v>90</v>
+        <v>191</v>
       </c>
       <c r="K315" t="s">
-        <v>90</v>
+        <v>191</v>
       </c>
       <c r="L315" t="s">
         <v>34</v>
@@ -20120,13 +20120,13 @@
         <v>47</v>
       </c>
       <c r="O315" t="s">
-        <v>310</v>
+        <v>34</v>
       </c>
       <c r="P315" t="s">
-        <v>667</v>
+        <v>34</v>
       </c>
       <c r="Q315" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="R315" t="s">
         <v>34</v>
@@ -20146,7 +20146,7 @@
         <v>34</v>
       </c>
       <c r="E316" t="s">
-        <v>244</v>
+        <v>223</v>
       </c>
       <c r="F316" t="s">
         <v>40</v>
@@ -20155,16 +20155,16 @@
         <v>41</v>
       </c>
       <c r="H316" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="I316" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="J316" t="s">
-        <v>119</v>
+        <v>147</v>
       </c>
       <c r="K316" t="s">
-        <v>80</v>
+        <v>113</v>
       </c>
       <c r="L316" t="s">
         <v>34</v>
@@ -20176,10 +20176,10 @@
         <v>47</v>
       </c>
       <c r="O316" t="s">
-        <v>247</v>
+        <v>114</v>
       </c>
       <c r="P316" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="Q316" t="s">
         <v>47</v>
@@ -20202,7 +20202,7 @@
         <v>34</v>
       </c>
       <c r="E317" t="s">
-        <v>248</v>
+        <v>275</v>
       </c>
       <c r="F317" t="s">
         <v>40</v>
@@ -20211,16 +20211,16 @@
         <v>41</v>
       </c>
       <c r="H317" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="I317" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="J317" t="s">
-        <v>119</v>
+        <v>96</v>
       </c>
       <c r="K317" t="s">
-        <v>119</v>
+        <v>58</v>
       </c>
       <c r="L317" t="s">
         <v>34</v>
@@ -20232,10 +20232,10 @@
         <v>47</v>
       </c>
       <c r="O317" t="s">
-        <v>250</v>
+        <v>105</v>
       </c>
       <c r="P317" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="Q317" t="s">
         <v>47</v>
@@ -20258,22 +20258,22 @@
         <v>34</v>
       </c>
       <c r="E318" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="F318" t="s">
-        <v>40</v>
+        <v>666</v>
       </c>
       <c r="G318" t="s">
         <v>41</v>
       </c>
       <c r="H318" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="I318" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="J318" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K318" t="s">
         <v>119</v>
@@ -20288,13 +20288,13 @@
         <v>47</v>
       </c>
       <c r="O318" t="s">
-        <v>130</v>
+        <v>34</v>
       </c>
       <c r="P318" t="s">
-        <v>667</v>
+        <v>34</v>
       </c>
       <c r="Q318" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="R318" t="s">
         <v>34</v>
@@ -20314,7 +20314,7 @@
         <v>34</v>
       </c>
       <c r="E319" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="F319" t="s">
         <v>40</v>
@@ -20323,16 +20323,16 @@
         <v>41</v>
       </c>
       <c r="H319" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="I319" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="J319" t="s">
-        <v>80</v>
+        <v>119</v>
       </c>
       <c r="K319" t="s">
-        <v>80</v>
+        <v>119</v>
       </c>
       <c r="L319" t="s">
         <v>34</v>
@@ -20344,10 +20344,10 @@
         <v>47</v>
       </c>
       <c r="O319" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="P319" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="Q319" t="s">
         <v>47</v>
@@ -20370,25 +20370,25 @@
         <v>34</v>
       </c>
       <c r="E320" t="s">
-        <v>227</v>
+        <v>157</v>
       </c>
       <c r="F320" t="s">
+        <v>40</v>
+      </c>
+      <c r="G320" t="s">
+        <v>41</v>
+      </c>
+      <c r="H320" t="s">
+        <v>667</v>
+      </c>
+      <c r="I320" t="s">
         <v>668</v>
       </c>
-      <c r="G320" t="s">
-        <v>41</v>
-      </c>
-      <c r="H320" t="s">
-        <v>666</v>
-      </c>
-      <c r="I320" t="s">
-        <v>667</v>
-      </c>
       <c r="J320" t="s">
-        <v>90</v>
+        <v>134</v>
       </c>
       <c r="K320" t="s">
-        <v>229</v>
+        <v>134</v>
       </c>
       <c r="L320" t="s">
         <v>34</v>
@@ -20400,13 +20400,13 @@
         <v>47</v>
       </c>
       <c r="O320" t="s">
-        <v>34</v>
+        <v>463</v>
       </c>
       <c r="P320" t="s">
-        <v>34</v>
+        <v>668</v>
       </c>
       <c r="Q320" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="R320" t="s">
         <v>34</v>
@@ -20426,25 +20426,25 @@
         <v>34</v>
       </c>
       <c r="E321" t="s">
-        <v>256</v>
+        <v>221</v>
       </c>
       <c r="F321" t="s">
+        <v>666</v>
+      </c>
+      <c r="G321" t="s">
+        <v>41</v>
+      </c>
+      <c r="H321" t="s">
+        <v>667</v>
+      </c>
+      <c r="I321" t="s">
         <v>668</v>
       </c>
-      <c r="G321" t="s">
-        <v>41</v>
-      </c>
-      <c r="H321" t="s">
-        <v>666</v>
-      </c>
-      <c r="I321" t="s">
-        <v>667</v>
-      </c>
       <c r="J321" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="K321" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="L321" t="s">
         <v>34</v>
@@ -20482,25 +20482,25 @@
         <v>34</v>
       </c>
       <c r="E322" t="s">
-        <v>236</v>
+        <v>253</v>
       </c>
       <c r="F322" t="s">
+        <v>40</v>
+      </c>
+      <c r="G322" t="s">
+        <v>41</v>
+      </c>
+      <c r="H322" t="s">
+        <v>667</v>
+      </c>
+      <c r="I322" t="s">
         <v>668</v>
       </c>
-      <c r="G322" t="s">
-        <v>41</v>
-      </c>
-      <c r="H322" t="s">
-        <v>666</v>
-      </c>
-      <c r="I322" t="s">
-        <v>667</v>
-      </c>
       <c r="J322" t="s">
-        <v>119</v>
+        <v>80</v>
       </c>
       <c r="K322" t="s">
-        <v>119</v>
+        <v>80</v>
       </c>
       <c r="L322" t="s">
         <v>34</v>
@@ -20512,13 +20512,13 @@
         <v>47</v>
       </c>
       <c r="O322" t="s">
-        <v>34</v>
+        <v>255</v>
       </c>
       <c r="P322" t="s">
-        <v>34</v>
+        <v>668</v>
       </c>
       <c r="Q322" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="R322" t="s">
         <v>34</v>
@@ -20538,7 +20538,7 @@
         <v>34</v>
       </c>
       <c r="E323" t="s">
-        <v>157</v>
+        <v>244</v>
       </c>
       <c r="F323" t="s">
         <v>40</v>
@@ -20547,16 +20547,16 @@
         <v>41</v>
       </c>
       <c r="H323" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="I323" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="J323" t="s">
-        <v>134</v>
+        <v>119</v>
       </c>
       <c r="K323" t="s">
-        <v>134</v>
+        <v>80</v>
       </c>
       <c r="L323" t="s">
         <v>34</v>
@@ -20568,10 +20568,10 @@
         <v>47</v>
       </c>
       <c r="O323" t="s">
-        <v>463</v>
+        <v>247</v>
       </c>
       <c r="P323" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="Q323" t="s">
         <v>47</v>
@@ -20594,7 +20594,7 @@
         <v>34</v>
       </c>
       <c r="E324" t="s">
-        <v>223</v>
+        <v>232</v>
       </c>
       <c r="F324" t="s">
         <v>40</v>
@@ -20603,16 +20603,16 @@
         <v>41</v>
       </c>
       <c r="H324" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="I324" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="J324" t="s">
-        <v>147</v>
+        <v>90</v>
       </c>
       <c r="K324" t="s">
-        <v>113</v>
+        <v>90</v>
       </c>
       <c r="L324" t="s">
         <v>34</v>
@@ -20624,10 +20624,10 @@
         <v>47</v>
       </c>
       <c r="O324" t="s">
-        <v>114</v>
+        <v>310</v>
       </c>
       <c r="P324" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="Q324" t="s">
         <v>47</v>
@@ -20650,7 +20650,7 @@
         <v>34</v>
       </c>
       <c r="E325" t="s">
-        <v>275</v>
+        <v>225</v>
       </c>
       <c r="F325" t="s">
         <v>40</v>
@@ -20659,16 +20659,16 @@
         <v>41</v>
       </c>
       <c r="H325" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="I325" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="J325" t="s">
-        <v>96</v>
+        <v>178</v>
       </c>
       <c r="K325" t="s">
-        <v>58</v>
+        <v>101</v>
       </c>
       <c r="L325" t="s">
         <v>34</v>
@@ -20680,10 +20680,10 @@
         <v>47</v>
       </c>
       <c r="O325" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="P325" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="Q325" t="s">
         <v>47</v>
@@ -20706,25 +20706,25 @@
         <v>34</v>
       </c>
       <c r="E326" t="s">
-        <v>221</v>
+        <v>256</v>
       </c>
       <c r="F326" t="s">
+        <v>666</v>
+      </c>
+      <c r="G326" t="s">
+        <v>41</v>
+      </c>
+      <c r="H326" t="s">
+        <v>667</v>
+      </c>
+      <c r="I326" t="s">
         <v>668</v>
       </c>
-      <c r="G326" t="s">
-        <v>41</v>
-      </c>
-      <c r="H326" t="s">
-        <v>666</v>
-      </c>
-      <c r="I326" t="s">
-        <v>667</v>
-      </c>
       <c r="J326" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="K326" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="L326" t="s">
         <v>34</v>
@@ -20762,25 +20762,25 @@
         <v>34</v>
       </c>
       <c r="E327" t="s">
-        <v>217</v>
+        <v>234</v>
       </c>
       <c r="F327" t="s">
+        <v>40</v>
+      </c>
+      <c r="G327" t="s">
+        <v>41</v>
+      </c>
+      <c r="H327" t="s">
+        <v>667</v>
+      </c>
+      <c r="I327" t="s">
         <v>668</v>
       </c>
-      <c r="G327" t="s">
-        <v>41</v>
-      </c>
-      <c r="H327" t="s">
-        <v>666</v>
-      </c>
-      <c r="I327" t="s">
-        <v>667</v>
-      </c>
       <c r="J327" t="s">
-        <v>191</v>
+        <v>118</v>
       </c>
       <c r="K327" t="s">
-        <v>191</v>
+        <v>119</v>
       </c>
       <c r="L327" t="s">
         <v>34</v>
@@ -20792,13 +20792,13 @@
         <v>47</v>
       </c>
       <c r="O327" t="s">
-        <v>34</v>
+        <v>130</v>
       </c>
       <c r="P327" t="s">
-        <v>34</v>
+        <v>668</v>
       </c>
       <c r="Q327" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="R327" t="s">
         <v>34</v>
@@ -20818,25 +20818,25 @@
         <v>34</v>
       </c>
       <c r="E328" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="F328" t="s">
-        <v>40</v>
+        <v>666</v>
       </c>
       <c r="G328" t="s">
         <v>41</v>
       </c>
       <c r="H328" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="I328" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="J328" t="s">
-        <v>178</v>
+        <v>90</v>
       </c>
       <c r="K328" t="s">
-        <v>101</v>
+        <v>229</v>
       </c>
       <c r="L328" t="s">
         <v>34</v>
@@ -20848,13 +20848,13 @@
         <v>47</v>
       </c>
       <c r="O328" t="s">
-        <v>102</v>
+        <v>34</v>
       </c>
       <c r="P328" t="s">
-        <v>667</v>
+        <v>34</v>
       </c>
       <c r="Q328" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="R328" t="s">
         <v>34</v>
@@ -20986,28 +20986,28 @@
         <v>34</v>
       </c>
       <c r="E331" t="s">
-        <v>175</v>
+        <v>676</v>
       </c>
       <c r="F331" t="s">
-        <v>40</v>
+        <v>211</v>
       </c>
       <c r="G331" t="s">
         <v>41</v>
       </c>
       <c r="H331" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="I331" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="J331" t="s">
-        <v>178</v>
+        <v>679</v>
       </c>
       <c r="K331" t="s">
-        <v>178</v>
+        <v>229</v>
       </c>
       <c r="L331" t="s">
-        <v>678</v>
+        <v>34</v>
       </c>
       <c r="M331" t="s">
         <v>671</v>
@@ -21019,7 +21019,7 @@
         <v>48</v>
       </c>
       <c r="P331" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="Q331" t="s">
         <v>47</v>
@@ -21042,7 +21042,7 @@
         <v>34</v>
       </c>
       <c r="E332" t="s">
-        <v>672</v>
+        <v>175</v>
       </c>
       <c r="F332" t="s">
         <v>40</v>
@@ -21051,16 +21051,16 @@
         <v>41</v>
       </c>
       <c r="H332" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="I332" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="J332" t="s">
-        <v>681</v>
+        <v>178</v>
       </c>
       <c r="K332" t="s">
-        <v>229</v>
+        <v>178</v>
       </c>
       <c r="L332" t="s">
         <v>682</v>
@@ -21075,7 +21075,7 @@
         <v>48</v>
       </c>
       <c r="P332" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="Q332" t="s">
         <v>47</v>
@@ -21098,28 +21098,28 @@
         <v>34</v>
       </c>
       <c r="E333" t="s">
+        <v>672</v>
+      </c>
+      <c r="F333" t="s">
+        <v>40</v>
+      </c>
+      <c r="G333" t="s">
+        <v>41</v>
+      </c>
+      <c r="H333" t="s">
         <v>683</v>
       </c>
-      <c r="F333" t="s">
-        <v>211</v>
-      </c>
-      <c r="G333" t="s">
-        <v>41</v>
-      </c>
-      <c r="H333" t="s">
+      <c r="I333" t="s">
         <v>684</v>
       </c>
-      <c r="I333" t="s">
+      <c r="J333" t="s">
         <v>685</v>
-      </c>
-      <c r="J333" t="s">
-        <v>686</v>
       </c>
       <c r="K333" t="s">
         <v>229</v>
       </c>
       <c r="L333" t="s">
-        <v>34</v>
+        <v>686</v>
       </c>
       <c r="M333" t="s">
         <v>671</v>
@@ -21131,7 +21131,7 @@
         <v>48</v>
       </c>
       <c r="P333" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="Q333" t="s">
         <v>47</v>
@@ -21337,7 +21337,7 @@
         <v>694</v>
       </c>
       <c r="J337" t="s">
-        <v>681</v>
+        <v>685</v>
       </c>
       <c r="K337" t="s">
         <v>45</v>
@@ -21490,7 +21490,7 @@
         <v>33</v>
       </c>
       <c r="E340" t="s">
-        <v>672</v>
+        <v>175</v>
       </c>
       <c r="F340" t="s">
         <v>40</v>
@@ -21499,13 +21499,13 @@
         <v>41</v>
       </c>
       <c r="H340" t="s">
-        <v>457</v>
+        <v>447</v>
       </c>
       <c r="I340" t="s">
-        <v>694</v>
+        <v>155</v>
       </c>
       <c r="J340" t="s">
-        <v>335</v>
+        <v>122</v>
       </c>
       <c r="K340" t="s">
         <v>45</v>
@@ -21523,7 +21523,7 @@
         <v>48</v>
       </c>
       <c r="P340" t="s">
-        <v>694</v>
+        <v>155</v>
       </c>
       <c r="Q340" t="s">
         <v>47</v>
@@ -21555,19 +21555,19 @@
         <v>41</v>
       </c>
       <c r="H341" t="s">
-        <v>556</v>
+        <v>215</v>
       </c>
       <c r="I341" t="s">
-        <v>694</v>
+        <v>704</v>
       </c>
       <c r="J341" t="s">
         <v>474</v>
       </c>
       <c r="K341" t="s">
-        <v>122</v>
+        <v>80</v>
       </c>
       <c r="L341" t="s">
-        <v>34</v>
+        <v>705</v>
       </c>
       <c r="M341" t="s">
         <v>701</v>
@@ -21579,7 +21579,7 @@
         <v>48</v>
       </c>
       <c r="P341" t="s">
-        <v>694</v>
+        <v>704</v>
       </c>
       <c r="Q341" t="s">
         <v>47</v>
@@ -21602,25 +21602,25 @@
         <v>34</v>
       </c>
       <c r="E342" t="s">
-        <v>704</v>
+        <v>175</v>
       </c>
       <c r="F342" t="s">
-        <v>211</v>
+        <v>40</v>
       </c>
       <c r="G342" t="s">
         <v>41</v>
       </c>
       <c r="H342" t="s">
-        <v>215</v>
+        <v>513</v>
       </c>
       <c r="I342" t="s">
-        <v>705</v>
+        <v>694</v>
       </c>
       <c r="J342" t="s">
-        <v>474</v>
+        <v>70</v>
       </c>
       <c r="K342" t="s">
-        <v>80</v>
+        <v>45</v>
       </c>
       <c r="L342" t="s">
         <v>706</v>
@@ -21635,7 +21635,7 @@
         <v>48</v>
       </c>
       <c r="P342" t="s">
-        <v>705</v>
+        <v>694</v>
       </c>
       <c r="Q342" t="s">
         <v>47</v>
@@ -21658,7 +21658,7 @@
         <v>34</v>
       </c>
       <c r="E343" t="s">
-        <v>175</v>
+        <v>672</v>
       </c>
       <c r="F343" t="s">
         <v>40</v>
@@ -21667,19 +21667,19 @@
         <v>41</v>
       </c>
       <c r="H343" t="s">
-        <v>511</v>
+        <v>707</v>
       </c>
       <c r="I343" t="s">
-        <v>694</v>
+        <v>708</v>
       </c>
       <c r="J343" t="s">
-        <v>70</v>
+        <v>685</v>
       </c>
       <c r="K343" t="s">
         <v>45</v>
       </c>
       <c r="L343" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
       <c r="M343" t="s">
         <v>701</v>
@@ -21691,7 +21691,7 @@
         <v>48</v>
       </c>
       <c r="P343" t="s">
-        <v>694</v>
+        <v>708</v>
       </c>
       <c r="Q343" t="s">
         <v>47</v>
@@ -21723,19 +21723,19 @@
         <v>41</v>
       </c>
       <c r="H344" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="I344" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
       <c r="J344" t="s">
-        <v>681</v>
+        <v>685</v>
       </c>
       <c r="K344" t="s">
         <v>45</v>
       </c>
       <c r="L344" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="M344" t="s">
         <v>701</v>
@@ -21747,7 +21747,7 @@
         <v>48</v>
       </c>
       <c r="P344" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
       <c r="Q344" t="s">
         <v>47</v>
@@ -21779,19 +21779,19 @@
         <v>41</v>
       </c>
       <c r="H345" t="s">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="I345" t="s">
-        <v>712</v>
+        <v>714</v>
       </c>
       <c r="J345" t="s">
-        <v>681</v>
+        <v>335</v>
       </c>
       <c r="K345" t="s">
         <v>45</v>
       </c>
       <c r="L345" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="M345" t="s">
         <v>701</v>
@@ -21803,7 +21803,7 @@
         <v>48</v>
       </c>
       <c r="P345" t="s">
-        <v>712</v>
+        <v>714</v>
       </c>
       <c r="Q345" t="s">
         <v>47</v>
@@ -21835,19 +21835,19 @@
         <v>41</v>
       </c>
       <c r="H346" t="s">
-        <v>714</v>
+        <v>459</v>
       </c>
       <c r="I346" t="s">
-        <v>694</v>
+        <v>708</v>
       </c>
       <c r="J346" t="s">
-        <v>681</v>
+        <v>685</v>
       </c>
       <c r="K346" t="s">
         <v>45</v>
       </c>
       <c r="L346" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="M346" t="s">
         <v>701</v>
@@ -21859,7 +21859,7 @@
         <v>48</v>
       </c>
       <c r="P346" t="s">
-        <v>694</v>
+        <v>708</v>
       </c>
       <c r="Q346" t="s">
         <v>47</v>
@@ -21891,19 +21891,19 @@
         <v>41</v>
       </c>
       <c r="H347" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="I347" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="J347" t="s">
-        <v>681</v>
+        <v>685</v>
       </c>
       <c r="K347" t="s">
         <v>45</v>
       </c>
       <c r="L347" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="M347" t="s">
         <v>701</v>
@@ -21915,7 +21915,7 @@
         <v>48</v>
       </c>
       <c r="P347" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="Q347" t="s">
         <v>47</v>
@@ -21947,10 +21947,10 @@
         <v>41</v>
       </c>
       <c r="H348" t="s">
-        <v>719</v>
+        <v>457</v>
       </c>
       <c r="I348" t="s">
-        <v>720</v>
+        <v>694</v>
       </c>
       <c r="J348" t="s">
         <v>335</v>
@@ -21959,7 +21959,7 @@
         <v>45</v>
       </c>
       <c r="L348" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="M348" t="s">
         <v>701</v>
@@ -21971,7 +21971,7 @@
         <v>48</v>
       </c>
       <c r="P348" t="s">
-        <v>720</v>
+        <v>694</v>
       </c>
       <c r="Q348" t="s">
         <v>47</v>
@@ -21994,28 +21994,28 @@
         <v>34</v>
       </c>
       <c r="E349" t="s">
-        <v>672</v>
+        <v>721</v>
       </c>
       <c r="F349" t="s">
-        <v>40</v>
+        <v>211</v>
       </c>
       <c r="G349" t="s">
         <v>41</v>
       </c>
       <c r="H349" t="s">
-        <v>459</v>
+        <v>556</v>
       </c>
       <c r="I349" t="s">
-        <v>722</v>
+        <v>694</v>
       </c>
       <c r="J349" t="s">
-        <v>681</v>
+        <v>474</v>
       </c>
       <c r="K349" t="s">
-        <v>45</v>
+        <v>122</v>
       </c>
       <c r="L349" t="s">
-        <v>723</v>
+        <v>34</v>
       </c>
       <c r="M349" t="s">
         <v>701</v>
@@ -22027,7 +22027,7 @@
         <v>48</v>
       </c>
       <c r="P349" t="s">
-        <v>722</v>
+        <v>694</v>
       </c>
       <c r="Q349" t="s">
         <v>47</v>
@@ -22059,7 +22059,7 @@
         <v>41</v>
       </c>
       <c r="H350" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="I350" t="s">
         <v>155</v>
@@ -22071,7 +22071,7 @@
         <v>122</v>
       </c>
       <c r="L350" t="s">
-        <v>725</v>
+        <v>723</v>
       </c>
       <c r="M350" t="s">
         <v>701</v>
@@ -22106,7 +22106,7 @@
         <v>34</v>
       </c>
       <c r="E351" t="s">
-        <v>175</v>
+        <v>672</v>
       </c>
       <c r="F351" t="s">
         <v>40</v>
@@ -22115,19 +22115,19 @@
         <v>41</v>
       </c>
       <c r="H351" t="s">
-        <v>447</v>
+        <v>724</v>
       </c>
       <c r="I351" t="s">
-        <v>155</v>
+        <v>694</v>
       </c>
       <c r="J351" t="s">
-        <v>122</v>
+        <v>685</v>
       </c>
       <c r="K351" t="s">
         <v>45</v>
       </c>
       <c r="L351" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="M351" t="s">
         <v>701</v>
@@ -22139,7 +22139,7 @@
         <v>48</v>
       </c>
       <c r="P351" t="s">
-        <v>155</v>
+        <v>694</v>
       </c>
       <c r="Q351" t="s">
         <v>47</v>
@@ -22162,7 +22162,7 @@
         <v>34</v>
       </c>
       <c r="E352" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="F352" t="s">
         <v>211</v>
@@ -22174,7 +22174,7 @@
         <v>425</v>
       </c>
       <c r="I352" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="J352" t="s">
         <v>474</v>
@@ -22195,7 +22195,7 @@
         <v>48</v>
       </c>
       <c r="P352" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="Q352" t="s">
         <v>47</v>
@@ -22227,13 +22227,13 @@
         <v>41</v>
       </c>
       <c r="H353" t="s">
+        <v>728</v>
+      </c>
+      <c r="I353" t="s">
         <v>729</v>
       </c>
-      <c r="I353" t="s">
-        <v>722</v>
-      </c>
       <c r="J353" t="s">
-        <v>681</v>
+        <v>685</v>
       </c>
       <c r="K353" t="s">
         <v>45</v>
@@ -22251,7 +22251,7 @@
         <v>48</v>
       </c>
       <c r="P353" t="s">
-        <v>722</v>
+        <v>729</v>
       </c>
       <c r="Q353" t="s">
         <v>47</v>
@@ -22669,7 +22669,7 @@
         <v>187</v>
       </c>
       <c r="F361" t="s">
-        <v>668</v>
+        <v>666</v>
       </c>
       <c r="G361" t="s">
         <v>41</v>
@@ -22843,16 +22843,16 @@
         <v>41</v>
       </c>
       <c r="H364" t="s">
-        <v>425</v>
+        <v>469</v>
       </c>
       <c r="I364" t="s">
         <v>754</v>
       </c>
       <c r="J364" t="s">
-        <v>178</v>
+        <v>101</v>
       </c>
       <c r="K364" t="s">
-        <v>178</v>
+        <v>101</v>
       </c>
       <c r="L364" t="s">
         <v>34</v>
@@ -22899,16 +22899,16 @@
         <v>41</v>
       </c>
       <c r="H365" t="s">
-        <v>469</v>
+        <v>425</v>
       </c>
       <c r="I365" t="s">
         <v>755</v>
       </c>
       <c r="J365" t="s">
-        <v>101</v>
+        <v>178</v>
       </c>
       <c r="K365" t="s">
-        <v>101</v>
+        <v>178</v>
       </c>
       <c r="L365" t="s">
         <v>34</v>
@@ -23073,7 +23073,7 @@
         <v>764</v>
       </c>
       <c r="J368" t="s">
-        <v>681</v>
+        <v>685</v>
       </c>
       <c r="K368" t="s">
         <v>229</v>
@@ -23353,7 +23353,7 @@
         <v>782</v>
       </c>
       <c r="J373" t="s">
-        <v>681</v>
+        <v>685</v>
       </c>
       <c r="K373" t="s">
         <v>45</v>
@@ -23521,7 +23521,7 @@
         <v>794</v>
       </c>
       <c r="J376" t="s">
-        <v>681</v>
+        <v>685</v>
       </c>
       <c r="K376" t="s">
         <v>795</v>
@@ -23692,7 +23692,7 @@
         <v>304</v>
       </c>
       <c r="K379" t="s">
-        <v>122</v>
+        <v>75</v>
       </c>
       <c r="L379" t="s">
         <v>805</v>
@@ -23739,19 +23739,19 @@
         <v>41</v>
       </c>
       <c r="H380" t="s">
+        <v>425</v>
+      </c>
+      <c r="I380" t="s">
         <v>807</v>
       </c>
-      <c r="I380" t="s">
+      <c r="J380" t="s">
+        <v>58</v>
+      </c>
+      <c r="K380" t="s">
+        <v>202</v>
+      </c>
+      <c r="L380" t="s">
         <v>808</v>
-      </c>
-      <c r="J380" t="s">
-        <v>304</v>
-      </c>
-      <c r="K380" t="s">
-        <v>96</v>
-      </c>
-      <c r="L380" t="s">
-        <v>809</v>
       </c>
       <c r="M380" t="s">
         <v>799</v>
@@ -23763,7 +23763,7 @@
         <v>48</v>
       </c>
       <c r="P380" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="Q380" t="s">
         <v>47</v>
@@ -23786,7 +23786,7 @@
         <v>34</v>
       </c>
       <c r="E381" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="F381" t="s">
         <v>211</v>
@@ -23795,10 +23795,10 @@
         <v>41</v>
       </c>
       <c r="H381" t="s">
+        <v>810</v>
+      </c>
+      <c r="I381" t="s">
         <v>811</v>
-      </c>
-      <c r="I381" t="s">
-        <v>812</v>
       </c>
       <c r="J381" t="s">
         <v>304</v>
@@ -23807,7 +23807,7 @@
         <v>96</v>
       </c>
       <c r="L381" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="M381" t="s">
         <v>799</v>
@@ -23819,7 +23819,7 @@
         <v>48</v>
       </c>
       <c r="P381" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="Q381" t="s">
         <v>47</v>
@@ -23842,7 +23842,7 @@
         <v>34</v>
       </c>
       <c r="E382" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="F382" t="s">
         <v>211</v>
@@ -23851,10 +23851,10 @@
         <v>41</v>
       </c>
       <c r="H382" t="s">
+        <v>814</v>
+      </c>
+      <c r="I382" t="s">
         <v>815</v>
-      </c>
-      <c r="I382" t="s">
-        <v>816</v>
       </c>
       <c r="J382" t="s">
         <v>304</v>
@@ -23863,7 +23863,7 @@
         <v>96</v>
       </c>
       <c r="L382" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="M382" t="s">
         <v>799</v>
@@ -23875,7 +23875,7 @@
         <v>48</v>
       </c>
       <c r="P382" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="Q382" t="s">
         <v>47</v>
@@ -23898,7 +23898,7 @@
         <v>34</v>
       </c>
       <c r="E383" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="F383" t="s">
         <v>211</v>
@@ -23907,7 +23907,7 @@
         <v>41</v>
       </c>
       <c r="H383" t="s">
-        <v>425</v>
+        <v>818</v>
       </c>
       <c r="I383" t="s">
         <v>819</v>
@@ -23972,7 +23972,7 @@
         <v>304</v>
       </c>
       <c r="K384" t="s">
-        <v>75</v>
+        <v>122</v>
       </c>
       <c r="L384" t="s">
         <v>824</v>
@@ -24025,10 +24025,10 @@
         <v>827</v>
       </c>
       <c r="J385" t="s">
-        <v>58</v>
+        <v>304</v>
       </c>
       <c r="K385" t="s">
-        <v>202</v>
+        <v>96</v>
       </c>
       <c r="L385" t="s">
         <v>828</v>
@@ -24137,7 +24137,7 @@
         <v>834</v>
       </c>
       <c r="J387" t="s">
-        <v>681</v>
+        <v>685</v>
       </c>
       <c r="K387" t="s">
         <v>45</v>
@@ -24346,28 +24346,28 @@
         <v>33</v>
       </c>
       <c r="E391" t="s">
+        <v>672</v>
+      </c>
+      <c r="F391" t="s">
+        <v>40</v>
+      </c>
+      <c r="G391" t="s">
+        <v>41</v>
+      </c>
+      <c r="H391" t="s">
         <v>850</v>
       </c>
-      <c r="F391" t="s">
-        <v>211</v>
-      </c>
-      <c r="G391" t="s">
-        <v>41</v>
-      </c>
-      <c r="H391" t="s">
+      <c r="I391" t="s">
         <v>851</v>
       </c>
-      <c r="I391" t="s">
+      <c r="J391" t="s">
+        <v>335</v>
+      </c>
+      <c r="K391" t="s">
+        <v>45</v>
+      </c>
+      <c r="L391" t="s">
         <v>852</v>
-      </c>
-      <c r="J391" t="s">
-        <v>304</v>
-      </c>
-      <c r="K391" t="s">
-        <v>122</v>
-      </c>
-      <c r="L391" t="s">
-        <v>34</v>
       </c>
       <c r="M391" t="s">
         <v>849</v>
@@ -24379,7 +24379,7 @@
         <v>48</v>
       </c>
       <c r="P391" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="Q391" t="s">
         <v>47</v>
@@ -24402,28 +24402,28 @@
         <v>34</v>
       </c>
       <c r="E392" t="s">
-        <v>672</v>
+        <v>853</v>
       </c>
       <c r="F392" t="s">
-        <v>40</v>
+        <v>211</v>
       </c>
       <c r="G392" t="s">
         <v>41</v>
       </c>
       <c r="H392" t="s">
-        <v>853</v>
+        <v>854</v>
       </c>
       <c r="I392" t="s">
-        <v>854</v>
+        <v>855</v>
       </c>
       <c r="J392" t="s">
-        <v>335</v>
+        <v>304</v>
       </c>
       <c r="K392" t="s">
-        <v>45</v>
+        <v>122</v>
       </c>
       <c r="L392" t="s">
-        <v>855</v>
+        <v>34</v>
       </c>
       <c r="M392" t="s">
         <v>849</v>
@@ -24435,7 +24435,7 @@
         <v>48</v>
       </c>
       <c r="P392" t="s">
-        <v>854</v>
+        <v>855</v>
       </c>
       <c r="Q392" t="s">
         <v>47</v>
@@ -24514,7 +24514,7 @@
         <v>34</v>
       </c>
       <c r="E394" t="s">
-        <v>860</v>
+        <v>672</v>
       </c>
       <c r="F394" t="s">
         <v>40</v>
@@ -24526,16 +24526,16 @@
         <v>845</v>
       </c>
       <c r="I394" t="s">
+        <v>860</v>
+      </c>
+      <c r="J394" t="s">
+        <v>335</v>
+      </c>
+      <c r="K394" t="s">
+        <v>858</v>
+      </c>
+      <c r="L394" t="s">
         <v>861</v>
-      </c>
-      <c r="J394" t="s">
-        <v>101</v>
-      </c>
-      <c r="K394" t="s">
-        <v>45</v>
-      </c>
-      <c r="L394" t="s">
-        <v>862</v>
       </c>
       <c r="M394" t="s">
         <v>849</v>
@@ -24547,7 +24547,7 @@
         <v>48</v>
       </c>
       <c r="P394" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="Q394" t="s">
         <v>47</v>
@@ -24570,7 +24570,7 @@
         <v>34</v>
       </c>
       <c r="E395" t="s">
-        <v>672</v>
+        <v>862</v>
       </c>
       <c r="F395" t="s">
         <v>40</v>
@@ -24585,10 +24585,10 @@
         <v>863</v>
       </c>
       <c r="J395" t="s">
-        <v>335</v>
+        <v>101</v>
       </c>
       <c r="K395" t="s">
-        <v>858</v>
+        <v>45</v>
       </c>
       <c r="L395" t="s">
         <v>864</v>
@@ -24809,7 +24809,7 @@
         <v>877</v>
       </c>
       <c r="J399" t="s">
-        <v>681</v>
+        <v>685</v>
       </c>
       <c r="K399" t="s">
         <v>45</v>
@@ -24862,7 +24862,7 @@
         <v>876</v>
       </c>
       <c r="I400" t="s">
-        <v>819</v>
+        <v>807</v>
       </c>
       <c r="J400" t="s">
         <v>58</v>
@@ -24883,7 +24883,7 @@
         <v>48</v>
       </c>
       <c r="P400" t="s">
-        <v>819</v>
+        <v>807</v>
       </c>
       <c r="Q400" t="s">
         <v>47</v>
@@ -25074,7 +25074,7 @@
         <v>33</v>
       </c>
       <c r="E404" t="s">
-        <v>672</v>
+        <v>762</v>
       </c>
       <c r="F404" t="s">
         <v>40</v>
@@ -25089,10 +25089,10 @@
         <v>897</v>
       </c>
       <c r="J404" t="s">
-        <v>681</v>
+        <v>178</v>
       </c>
       <c r="K404" t="s">
-        <v>45</v>
+        <v>178</v>
       </c>
       <c r="L404" t="s">
         <v>898</v>
@@ -25130,7 +25130,7 @@
         <v>34</v>
       </c>
       <c r="E405" t="s">
-        <v>762</v>
+        <v>672</v>
       </c>
       <c r="F405" t="s">
         <v>40</v>
@@ -25145,10 +25145,10 @@
         <v>900</v>
       </c>
       <c r="J405" t="s">
-        <v>178</v>
+        <v>685</v>
       </c>
       <c r="K405" t="s">
-        <v>178</v>
+        <v>45</v>
       </c>
       <c r="L405" t="s">
         <v>901</v>

</xml_diff>

<commit_message>
dados: 2026-10-19 08:22 (132 arquivos)
</commit_message>
<xml_diff>
--- a/xlsx/dre/DRE_02_2026.xlsx
+++ b/xlsx/dre/DRE_02_2026.xlsx
@@ -2028,15 +2028,15 @@
     <t>4.03.03.02.05.02 Assistência técnica medição</t>
   </si>
   <si>
+    <t>L E A Medicoes Tecnicas LTDA</t>
+  </si>
+  <si>
+    <t>R$  180,00</t>
+  </si>
+  <si>
     <t>PFP</t>
   </si>
   <si>
-    <t>L E A Medicoes Tecnicas LTDA</t>
-  </si>
-  <si>
-    <t>R$  180,00</t>
-  </si>
-  <si>
     <t>4.03.03.09 Marketing - mídias / ações comerciais / outros (CV)</t>
   </si>
   <si>
@@ -2058,6 +2058,27 @@
     <t>Google 2026</t>
   </si>
   <si>
+    <t>WEBGIGA SOLUCOES DIGITAIS LTDA</t>
+  </si>
+  <si>
+    <t>R$  4.588,50</t>
+  </si>
+  <si>
+    <t>Webgiga 2026</t>
+  </si>
+  <si>
+    <t>MARQUES MAIO MARKETING DIGITAL LTDA</t>
+  </si>
+  <si>
+    <t>R$  808,50</t>
+  </si>
+  <si>
+    <t>08/01/26</t>
+  </si>
+  <si>
+    <t>MHM - Honorários 2026</t>
+  </si>
+  <si>
     <t>498/1</t>
   </si>
   <si>
@@ -2070,27 +2091,6 @@
     <t>30/01/26</t>
   </si>
   <si>
-    <t>WEBGIGA SOLUCOES DIGITAIS LTDA</t>
-  </si>
-  <si>
-    <t>R$  4.588,50</t>
-  </si>
-  <si>
-    <t>Webgiga 2026</t>
-  </si>
-  <si>
-    <t>MARQUES MAIO MARKETING DIGITAL LTDA</t>
-  </si>
-  <si>
-    <t>R$  808,50</t>
-  </si>
-  <si>
-    <t>08/01/26</t>
-  </si>
-  <si>
-    <t>MHM - Honorários 2026</t>
-  </si>
-  <si>
     <t>4.04 DESPESAS ADMINISTRATIVAS</t>
   </si>
   <si>
@@ -2295,12 +2295,12 @@
     <t>VT fev 26/1</t>
   </si>
   <si>
+    <t>R$  313,70</t>
+  </si>
+  <si>
     <t>R$  433,98</t>
   </si>
   <si>
-    <t>R$  313,70</t>
-  </si>
-  <si>
     <t>4.04.02 GASTOS GERAIS ADMINISTRATIVOS</t>
   </si>
   <si>
@@ -2439,25 +2439,17 @@
     <t>R$  45,00</t>
   </si>
   <si>
-    <t>532/1</t>
-  </si>
-  <si>
-    <t>DIA BRASIL SUPERMERCADO</t>
-  </si>
-  <si>
-    <t>R$  59,96</t>
-  </si>
-  <si>
-    <t>cafés</t>
-  </si>
-  <si>
-    <t>502/1</t>
-  </si>
-  <si>
-    <t>R$  100,00</t>
-  </si>
-  <si>
-    <t>Cópia de chaves</t>
+    <t>531/1</t>
+  </si>
+  <si>
+    <t>Shopee</t>
+  </si>
+  <si>
+    <t>R$  65,93</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Freeco refil
+</t>
   </si>
   <si>
     <t>533/1</t>
@@ -2470,6 +2462,19 @@
   </si>
   <si>
     <t>material limpeza</t>
+  </si>
+  <si>
+    <t>530/1</t>
+  </si>
+  <si>
+    <t>Marinete</t>
+  </si>
+  <si>
+    <t>R$  17,00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Copo descartável para crianças
+</t>
   </si>
   <si>
     <t>529/1</t>
@@ -2486,6 +2491,27 @@
 </t>
   </si>
   <si>
+    <t>502/1</t>
+  </si>
+  <si>
+    <t>R$  100,00</t>
+  </si>
+  <si>
+    <t>Cópia de chaves</t>
+  </si>
+  <si>
+    <t>532/1</t>
+  </si>
+  <si>
+    <t>DIA BRASIL SUPERMERCADO</t>
+  </si>
+  <si>
+    <t>R$  59,96</t>
+  </si>
+  <si>
+    <t>cafés</t>
+  </si>
+  <si>
     <t>505/1</t>
   </si>
   <si>
@@ -2498,32 +2524,6 @@
     <t>Conserto vidro adega</t>
   </si>
   <si>
-    <t>531/1</t>
-  </si>
-  <si>
-    <t>Shopee</t>
-  </si>
-  <si>
-    <t>R$  65,93</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Freeco refil
-</t>
-  </si>
-  <si>
-    <t>530/1</t>
-  </si>
-  <si>
-    <t>Marinete</t>
-  </si>
-  <si>
-    <t>R$  17,00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Copo descartável para crianças
-</t>
-  </si>
-  <si>
     <t>4.04.02.07 Informática</t>
   </si>
   <si>
@@ -2587,6 +2587,15 @@
     <t>4.04.02.08.03 Mensalidades e assinaturas - outros gastos</t>
   </si>
   <si>
+    <t>534/1</t>
+  </si>
+  <si>
+    <t>Pipefy</t>
+  </si>
+  <si>
+    <t>R$  197,63</t>
+  </si>
+  <si>
     <t>D4 sign</t>
   </si>
   <si>
@@ -2596,15 +2605,6 @@
     <t>D4 sign 2026</t>
   </si>
   <si>
-    <t>534/1</t>
-  </si>
-  <si>
-    <t>Pipefy</t>
-  </si>
-  <si>
-    <t>R$  197,63</t>
-  </si>
-  <si>
     <t>10/2</t>
   </si>
   <si>
@@ -2617,19 +2617,19 @@
     <t>Promob 2026-1</t>
   </si>
   <si>
+    <t>3/1</t>
+  </si>
+  <si>
+    <t>R$  1.248,76</t>
+  </si>
+  <si>
+    <t>Promob 2026/2</t>
+  </si>
+  <si>
     <t>R$  599,00</t>
   </si>
   <si>
     <t>Promob 2026</t>
-  </si>
-  <si>
-    <t>3/1</t>
-  </si>
-  <si>
-    <t>R$  1.248,76</t>
-  </si>
-  <si>
-    <t>Promob 2026/2</t>
   </si>
   <si>
     <t>4.04.02.11 Manutenção de predio e equipamentos</t>
@@ -2726,6 +2726,15 @@
     <t>R$ 400,33</t>
   </si>
   <si>
+    <t>Jackson Fernando de Araujo</t>
+  </si>
+  <si>
+    <t>R$  150,00</t>
+  </si>
+  <si>
+    <t>Segurança 2026</t>
+  </si>
+  <si>
     <t>VERISURE</t>
   </si>
   <si>
@@ -2733,15 +2742,6 @@
   </si>
   <si>
     <t>Verisure - Alarme 2026</t>
-  </si>
-  <si>
-    <t>Jackson Fernando de Araujo</t>
-  </si>
-  <si>
-    <t>R$  150,00</t>
-  </si>
-  <si>
-    <t>Segurança 2026</t>
   </si>
   <si>
     <t>4.04.02.14.08 Site e newsletter da loja</t>
@@ -20093,25 +20093,25 @@
         <v>33</v>
       </c>
       <c r="E315" t="s">
-        <v>217</v>
+        <v>232</v>
       </c>
       <c r="F315" t="s">
+        <v>40</v>
+      </c>
+      <c r="G315" t="s">
+        <v>41</v>
+      </c>
+      <c r="H315" t="s">
         <v>666</v>
       </c>
-      <c r="G315" t="s">
-        <v>41</v>
-      </c>
-      <c r="H315" t="s">
+      <c r="I315" t="s">
         <v>667</v>
       </c>
-      <c r="I315" t="s">
-        <v>668</v>
-      </c>
       <c r="J315" t="s">
-        <v>191</v>
+        <v>90</v>
       </c>
       <c r="K315" t="s">
-        <v>191</v>
+        <v>90</v>
       </c>
       <c r="L315" t="s">
         <v>34</v>
@@ -20123,13 +20123,13 @@
         <v>47</v>
       </c>
       <c r="O315" t="s">
-        <v>34</v>
+        <v>308</v>
       </c>
       <c r="P315" t="s">
-        <v>34</v>
+        <v>667</v>
       </c>
       <c r="Q315" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="R315" t="s">
         <v>34</v>
@@ -20149,7 +20149,7 @@
         <v>34</v>
       </c>
       <c r="E316" t="s">
-        <v>223</v>
+        <v>244</v>
       </c>
       <c r="F316" t="s">
         <v>40</v>
@@ -20158,16 +20158,16 @@
         <v>41</v>
       </c>
       <c r="H316" t="s">
+        <v>666</v>
+      </c>
+      <c r="I316" t="s">
         <v>667</v>
       </c>
-      <c r="I316" t="s">
-        <v>668</v>
-      </c>
       <c r="J316" t="s">
-        <v>147</v>
+        <v>119</v>
       </c>
       <c r="K316" t="s">
-        <v>113</v>
+        <v>80</v>
       </c>
       <c r="L316" t="s">
         <v>34</v>
@@ -20179,10 +20179,10 @@
         <v>47</v>
       </c>
       <c r="O316" t="s">
-        <v>114</v>
+        <v>247</v>
       </c>
       <c r="P316" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="Q316" t="s">
         <v>47</v>
@@ -20205,7 +20205,7 @@
         <v>34</v>
       </c>
       <c r="E317" t="s">
-        <v>275</v>
+        <v>248</v>
       </c>
       <c r="F317" t="s">
         <v>40</v>
@@ -20214,16 +20214,16 @@
         <v>41</v>
       </c>
       <c r="H317" t="s">
+        <v>666</v>
+      </c>
+      <c r="I317" t="s">
         <v>667</v>
       </c>
-      <c r="I317" t="s">
-        <v>668</v>
-      </c>
       <c r="J317" t="s">
-        <v>96</v>
+        <v>119</v>
       </c>
       <c r="K317" t="s">
-        <v>58</v>
+        <v>119</v>
       </c>
       <c r="L317" t="s">
         <v>34</v>
@@ -20235,10 +20235,10 @@
         <v>47</v>
       </c>
       <c r="O317" t="s">
-        <v>105</v>
+        <v>250</v>
       </c>
       <c r="P317" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="Q317" t="s">
         <v>47</v>
@@ -20261,22 +20261,22 @@
         <v>34</v>
       </c>
       <c r="E318" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="F318" t="s">
+        <v>40</v>
+      </c>
+      <c r="G318" t="s">
+        <v>41</v>
+      </c>
+      <c r="H318" t="s">
         <v>666</v>
       </c>
-      <c r="G318" t="s">
-        <v>41</v>
-      </c>
-      <c r="H318" t="s">
+      <c r="I318" t="s">
         <v>667</v>
       </c>
-      <c r="I318" t="s">
-        <v>668</v>
-      </c>
       <c r="J318" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="K318" t="s">
         <v>119</v>
@@ -20291,13 +20291,13 @@
         <v>47</v>
       </c>
       <c r="O318" t="s">
-        <v>34</v>
+        <v>130</v>
       </c>
       <c r="P318" t="s">
-        <v>34</v>
+        <v>667</v>
       </c>
       <c r="Q318" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="R318" t="s">
         <v>34</v>
@@ -20317,7 +20317,7 @@
         <v>34</v>
       </c>
       <c r="E319" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="F319" t="s">
         <v>40</v>
@@ -20326,16 +20326,16 @@
         <v>41</v>
       </c>
       <c r="H319" t="s">
+        <v>666</v>
+      </c>
+      <c r="I319" t="s">
         <v>667</v>
       </c>
-      <c r="I319" t="s">
-        <v>668</v>
-      </c>
       <c r="J319" t="s">
-        <v>119</v>
+        <v>80</v>
       </c>
       <c r="K319" t="s">
-        <v>119</v>
+        <v>80</v>
       </c>
       <c r="L319" t="s">
         <v>34</v>
@@ -20347,10 +20347,10 @@
         <v>47</v>
       </c>
       <c r="O319" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="P319" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="Q319" t="s">
         <v>47</v>
@@ -20373,25 +20373,25 @@
         <v>34</v>
       </c>
       <c r="E320" t="s">
-        <v>157</v>
+        <v>227</v>
       </c>
       <c r="F320" t="s">
-        <v>40</v>
+        <v>668</v>
       </c>
       <c r="G320" t="s">
         <v>41</v>
       </c>
       <c r="H320" t="s">
+        <v>666</v>
+      </c>
+      <c r="I320" t="s">
         <v>667</v>
       </c>
-      <c r="I320" t="s">
-        <v>668</v>
-      </c>
       <c r="J320" t="s">
-        <v>134</v>
+        <v>90</v>
       </c>
       <c r="K320" t="s">
-        <v>134</v>
+        <v>229</v>
       </c>
       <c r="L320" t="s">
         <v>34</v>
@@ -20403,13 +20403,13 @@
         <v>47</v>
       </c>
       <c r="O320" t="s">
-        <v>463</v>
+        <v>34</v>
       </c>
       <c r="P320" t="s">
-        <v>668</v>
+        <v>34</v>
       </c>
       <c r="Q320" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="R320" t="s">
         <v>34</v>
@@ -20429,25 +20429,25 @@
         <v>34</v>
       </c>
       <c r="E321" t="s">
-        <v>221</v>
+        <v>256</v>
       </c>
       <c r="F321" t="s">
+        <v>668</v>
+      </c>
+      <c r="G321" t="s">
+        <v>41</v>
+      </c>
+      <c r="H321" t="s">
         <v>666</v>
       </c>
-      <c r="G321" t="s">
-        <v>41</v>
-      </c>
-      <c r="H321" t="s">
+      <c r="I321" t="s">
         <v>667</v>
       </c>
-      <c r="I321" t="s">
-        <v>668</v>
-      </c>
       <c r="J321" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="K321" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="L321" t="s">
         <v>34</v>
@@ -20485,25 +20485,25 @@
         <v>34</v>
       </c>
       <c r="E322" t="s">
-        <v>253</v>
+        <v>236</v>
       </c>
       <c r="F322" t="s">
-        <v>40</v>
+        <v>668</v>
       </c>
       <c r="G322" t="s">
         <v>41</v>
       </c>
       <c r="H322" t="s">
+        <v>666</v>
+      </c>
+      <c r="I322" t="s">
         <v>667</v>
       </c>
-      <c r="I322" t="s">
-        <v>668</v>
-      </c>
       <c r="J322" t="s">
-        <v>80</v>
+        <v>119</v>
       </c>
       <c r="K322" t="s">
-        <v>80</v>
+        <v>119</v>
       </c>
       <c r="L322" t="s">
         <v>34</v>
@@ -20515,13 +20515,13 @@
         <v>47</v>
       </c>
       <c r="O322" t="s">
-        <v>255</v>
+        <v>34</v>
       </c>
       <c r="P322" t="s">
-        <v>668</v>
+        <v>34</v>
       </c>
       <c r="Q322" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="R322" t="s">
         <v>34</v>
@@ -20541,7 +20541,7 @@
         <v>34</v>
       </c>
       <c r="E323" t="s">
-        <v>244</v>
+        <v>157</v>
       </c>
       <c r="F323" t="s">
         <v>40</v>
@@ -20550,16 +20550,16 @@
         <v>41</v>
       </c>
       <c r="H323" t="s">
+        <v>666</v>
+      </c>
+      <c r="I323" t="s">
         <v>667</v>
       </c>
-      <c r="I323" t="s">
-        <v>668</v>
-      </c>
       <c r="J323" t="s">
-        <v>119</v>
+        <v>134</v>
       </c>
       <c r="K323" t="s">
-        <v>80</v>
+        <v>134</v>
       </c>
       <c r="L323" t="s">
         <v>34</v>
@@ -20571,10 +20571,10 @@
         <v>47</v>
       </c>
       <c r="O323" t="s">
-        <v>247</v>
+        <v>463</v>
       </c>
       <c r="P323" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="Q323" t="s">
         <v>47</v>
@@ -20597,7 +20597,7 @@
         <v>34</v>
       </c>
       <c r="E324" t="s">
-        <v>232</v>
+        <v>223</v>
       </c>
       <c r="F324" t="s">
         <v>40</v>
@@ -20606,16 +20606,16 @@
         <v>41</v>
       </c>
       <c r="H324" t="s">
+        <v>666</v>
+      </c>
+      <c r="I324" t="s">
         <v>667</v>
       </c>
-      <c r="I324" t="s">
-        <v>668</v>
-      </c>
       <c r="J324" t="s">
-        <v>90</v>
+        <v>147</v>
       </c>
       <c r="K324" t="s">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="L324" t="s">
         <v>34</v>
@@ -20627,10 +20627,10 @@
         <v>47</v>
       </c>
       <c r="O324" t="s">
-        <v>308</v>
+        <v>114</v>
       </c>
       <c r="P324" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="Q324" t="s">
         <v>47</v>
@@ -20653,7 +20653,7 @@
         <v>34</v>
       </c>
       <c r="E325" t="s">
-        <v>225</v>
+        <v>275</v>
       </c>
       <c r="F325" t="s">
         <v>40</v>
@@ -20662,16 +20662,16 @@
         <v>41</v>
       </c>
       <c r="H325" t="s">
+        <v>666</v>
+      </c>
+      <c r="I325" t="s">
         <v>667</v>
       </c>
-      <c r="I325" t="s">
-        <v>668</v>
-      </c>
       <c r="J325" t="s">
-        <v>178</v>
+        <v>96</v>
       </c>
       <c r="K325" t="s">
-        <v>101</v>
+        <v>58</v>
       </c>
       <c r="L325" t="s">
         <v>34</v>
@@ -20683,10 +20683,10 @@
         <v>47</v>
       </c>
       <c r="O325" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="P325" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="Q325" t="s">
         <v>47</v>
@@ -20709,25 +20709,25 @@
         <v>34</v>
       </c>
       <c r="E326" t="s">
-        <v>256</v>
+        <v>221</v>
       </c>
       <c r="F326" t="s">
+        <v>668</v>
+      </c>
+      <c r="G326" t="s">
+        <v>41</v>
+      </c>
+      <c r="H326" t="s">
         <v>666</v>
       </c>
-      <c r="G326" t="s">
-        <v>41</v>
-      </c>
-      <c r="H326" t="s">
+      <c r="I326" t="s">
         <v>667</v>
       </c>
-      <c r="I326" t="s">
-        <v>668</v>
-      </c>
       <c r="J326" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="K326" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="L326" t="s">
         <v>34</v>
@@ -20765,25 +20765,25 @@
         <v>34</v>
       </c>
       <c r="E327" t="s">
-        <v>234</v>
+        <v>217</v>
       </c>
       <c r="F327" t="s">
-        <v>40</v>
+        <v>668</v>
       </c>
       <c r="G327" t="s">
         <v>41</v>
       </c>
       <c r="H327" t="s">
+        <v>666</v>
+      </c>
+      <c r="I327" t="s">
         <v>667</v>
       </c>
-      <c r="I327" t="s">
-        <v>668</v>
-      </c>
       <c r="J327" t="s">
-        <v>118</v>
+        <v>191</v>
       </c>
       <c r="K327" t="s">
-        <v>119</v>
+        <v>191</v>
       </c>
       <c r="L327" t="s">
         <v>34</v>
@@ -20795,13 +20795,13 @@
         <v>47</v>
       </c>
       <c r="O327" t="s">
-        <v>130</v>
+        <v>34</v>
       </c>
       <c r="P327" t="s">
-        <v>668</v>
+        <v>34</v>
       </c>
       <c r="Q327" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="R327" t="s">
         <v>34</v>
@@ -20821,25 +20821,25 @@
         <v>34</v>
       </c>
       <c r="E328" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="F328" t="s">
+        <v>40</v>
+      </c>
+      <c r="G328" t="s">
+        <v>41</v>
+      </c>
+      <c r="H328" t="s">
         <v>666</v>
       </c>
-      <c r="G328" t="s">
-        <v>41</v>
-      </c>
-      <c r="H328" t="s">
+      <c r="I328" t="s">
         <v>667</v>
       </c>
-      <c r="I328" t="s">
-        <v>668</v>
-      </c>
       <c r="J328" t="s">
-        <v>90</v>
+        <v>178</v>
       </c>
       <c r="K328" t="s">
-        <v>229</v>
+        <v>101</v>
       </c>
       <c r="L328" t="s">
         <v>34</v>
@@ -20851,13 +20851,13 @@
         <v>47</v>
       </c>
       <c r="O328" t="s">
-        <v>34</v>
+        <v>102</v>
       </c>
       <c r="P328" t="s">
-        <v>34</v>
+        <v>667</v>
       </c>
       <c r="Q328" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="R328" t="s">
         <v>34</v>
@@ -20989,28 +20989,28 @@
         <v>34</v>
       </c>
       <c r="E331" t="s">
+        <v>175</v>
+      </c>
+      <c r="F331" t="s">
+        <v>40</v>
+      </c>
+      <c r="G331" t="s">
+        <v>41</v>
+      </c>
+      <c r="H331" t="s">
         <v>676</v>
       </c>
-      <c r="F331" t="s">
-        <v>211</v>
-      </c>
-      <c r="G331" t="s">
-        <v>41</v>
-      </c>
-      <c r="H331" t="s">
+      <c r="I331" t="s">
         <v>677</v>
       </c>
-      <c r="I331" t="s">
+      <c r="J331" t="s">
+        <v>178</v>
+      </c>
+      <c r="K331" t="s">
+        <v>178</v>
+      </c>
+      <c r="L331" t="s">
         <v>678</v>
-      </c>
-      <c r="J331" t="s">
-        <v>679</v>
-      </c>
-      <c r="K331" t="s">
-        <v>229</v>
-      </c>
-      <c r="L331" t="s">
-        <v>34</v>
       </c>
       <c r="M331" t="s">
         <v>671</v>
@@ -21022,7 +21022,7 @@
         <v>48</v>
       </c>
       <c r="P331" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="Q331" t="s">
         <v>47</v>
@@ -21045,7 +21045,7 @@
         <v>34</v>
       </c>
       <c r="E332" t="s">
-        <v>175</v>
+        <v>672</v>
       </c>
       <c r="F332" t="s">
         <v>40</v>
@@ -21054,16 +21054,16 @@
         <v>41</v>
       </c>
       <c r="H332" t="s">
+        <v>679</v>
+      </c>
+      <c r="I332" t="s">
         <v>680</v>
       </c>
-      <c r="I332" t="s">
+      <c r="J332" t="s">
         <v>681</v>
       </c>
-      <c r="J332" t="s">
-        <v>178</v>
-      </c>
       <c r="K332" t="s">
-        <v>178</v>
+        <v>229</v>
       </c>
       <c r="L332" t="s">
         <v>682</v>
@@ -21078,7 +21078,7 @@
         <v>48</v>
       </c>
       <c r="P332" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="Q332" t="s">
         <v>47</v>
@@ -21101,28 +21101,28 @@
         <v>34</v>
       </c>
       <c r="E333" t="s">
-        <v>672</v>
+        <v>683</v>
       </c>
       <c r="F333" t="s">
-        <v>40</v>
+        <v>211</v>
       </c>
       <c r="G333" t="s">
         <v>41</v>
       </c>
       <c r="H333" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="I333" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="J333" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="K333" t="s">
         <v>229</v>
       </c>
       <c r="L333" t="s">
-        <v>686</v>
+        <v>34</v>
       </c>
       <c r="M333" t="s">
         <v>671</v>
@@ -21134,7 +21134,7 @@
         <v>48</v>
       </c>
       <c r="P333" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="Q333" t="s">
         <v>47</v>
@@ -21340,7 +21340,7 @@
         <v>694</v>
       </c>
       <c r="J337" t="s">
-        <v>685</v>
+        <v>681</v>
       </c>
       <c r="K337" t="s">
         <v>45</v>
@@ -21508,7 +21508,7 @@
         <v>703</v>
       </c>
       <c r="J340" t="s">
-        <v>685</v>
+        <v>681</v>
       </c>
       <c r="K340" t="s">
         <v>45</v>
@@ -21564,7 +21564,7 @@
         <v>706</v>
       </c>
       <c r="J341" t="s">
-        <v>685</v>
+        <v>681</v>
       </c>
       <c r="K341" t="s">
         <v>45</v>
@@ -21676,7 +21676,7 @@
         <v>694</v>
       </c>
       <c r="J343" t="s">
-        <v>685</v>
+        <v>681</v>
       </c>
       <c r="K343" t="s">
         <v>45</v>
@@ -21732,7 +21732,7 @@
         <v>712</v>
       </c>
       <c r="J344" t="s">
-        <v>685</v>
+        <v>681</v>
       </c>
       <c r="K344" t="s">
         <v>45</v>
@@ -21788,7 +21788,7 @@
         <v>715</v>
       </c>
       <c r="J345" t="s">
-        <v>685</v>
+        <v>681</v>
       </c>
       <c r="K345" t="s">
         <v>45</v>
@@ -21900,7 +21900,7 @@
         <v>715</v>
       </c>
       <c r="J347" t="s">
-        <v>685</v>
+        <v>681</v>
       </c>
       <c r="K347" t="s">
         <v>45</v>
@@ -22672,7 +22672,7 @@
         <v>187</v>
       </c>
       <c r="F361" t="s">
-        <v>666</v>
+        <v>668</v>
       </c>
       <c r="G361" t="s">
         <v>41</v>
@@ -22846,16 +22846,16 @@
         <v>41</v>
       </c>
       <c r="H364" t="s">
-        <v>469</v>
+        <v>425</v>
       </c>
       <c r="I364" t="s">
         <v>755</v>
       </c>
       <c r="J364" t="s">
-        <v>101</v>
+        <v>178</v>
       </c>
       <c r="K364" t="s">
-        <v>101</v>
+        <v>178</v>
       </c>
       <c r="L364" t="s">
         <v>34</v>
@@ -22902,16 +22902,16 @@
         <v>41</v>
       </c>
       <c r="H365" t="s">
-        <v>425</v>
+        <v>469</v>
       </c>
       <c r="I365" t="s">
         <v>756</v>
       </c>
       <c r="J365" t="s">
-        <v>178</v>
+        <v>101</v>
       </c>
       <c r="K365" t="s">
-        <v>178</v>
+        <v>101</v>
       </c>
       <c r="L365" t="s">
         <v>34</v>
@@ -23076,7 +23076,7 @@
         <v>765</v>
       </c>
       <c r="J368" t="s">
-        <v>685</v>
+        <v>681</v>
       </c>
       <c r="K368" t="s">
         <v>229</v>
@@ -23356,7 +23356,7 @@
         <v>783</v>
       </c>
       <c r="J373" t="s">
-        <v>685</v>
+        <v>681</v>
       </c>
       <c r="K373" t="s">
         <v>45</v>
@@ -23524,7 +23524,7 @@
         <v>795</v>
       </c>
       <c r="J376" t="s">
-        <v>685</v>
+        <v>681</v>
       </c>
       <c r="K376" t="s">
         <v>796</v>
@@ -23695,7 +23695,7 @@
         <v>320</v>
       </c>
       <c r="K379" t="s">
-        <v>75</v>
+        <v>122</v>
       </c>
       <c r="L379" t="s">
         <v>806</v>
@@ -23742,19 +23742,19 @@
         <v>41</v>
       </c>
       <c r="H380" t="s">
-        <v>425</v>
+        <v>808</v>
       </c>
       <c r="I380" t="s">
-        <v>808</v>
+        <v>809</v>
       </c>
       <c r="J380" t="s">
-        <v>58</v>
+        <v>320</v>
       </c>
       <c r="K380" t="s">
-        <v>202</v>
+        <v>96</v>
       </c>
       <c r="L380" t="s">
-        <v>809</v>
+        <v>810</v>
       </c>
       <c r="M380" t="s">
         <v>800</v>
@@ -23766,7 +23766,7 @@
         <v>48</v>
       </c>
       <c r="P380" t="s">
-        <v>808</v>
+        <v>809</v>
       </c>
       <c r="Q380" t="s">
         <v>47</v>
@@ -23789,7 +23789,7 @@
         <v>34</v>
       </c>
       <c r="E381" t="s">
-        <v>810</v>
+        <v>811</v>
       </c>
       <c r="F381" t="s">
         <v>211</v>
@@ -23798,10 +23798,10 @@
         <v>41</v>
       </c>
       <c r="H381" t="s">
-        <v>811</v>
+        <v>812</v>
       </c>
       <c r="I381" t="s">
-        <v>812</v>
+        <v>813</v>
       </c>
       <c r="J381" t="s">
         <v>320</v>
@@ -23810,7 +23810,7 @@
         <v>96</v>
       </c>
       <c r="L381" t="s">
-        <v>813</v>
+        <v>814</v>
       </c>
       <c r="M381" t="s">
         <v>800</v>
@@ -23822,7 +23822,7 @@
         <v>48</v>
       </c>
       <c r="P381" t="s">
-        <v>812</v>
+        <v>813</v>
       </c>
       <c r="Q381" t="s">
         <v>47</v>
@@ -23845,7 +23845,7 @@
         <v>34</v>
       </c>
       <c r="E382" t="s">
-        <v>814</v>
+        <v>815</v>
       </c>
       <c r="F382" t="s">
         <v>211</v>
@@ -23854,10 +23854,10 @@
         <v>41</v>
       </c>
       <c r="H382" t="s">
-        <v>815</v>
+        <v>816</v>
       </c>
       <c r="I382" t="s">
-        <v>816</v>
+        <v>817</v>
       </c>
       <c r="J382" t="s">
         <v>320</v>
@@ -23866,7 +23866,7 @@
         <v>96</v>
       </c>
       <c r="L382" t="s">
-        <v>817</v>
+        <v>818</v>
       </c>
       <c r="M382" t="s">
         <v>800</v>
@@ -23878,7 +23878,7 @@
         <v>48</v>
       </c>
       <c r="P382" t="s">
-        <v>816</v>
+        <v>817</v>
       </c>
       <c r="Q382" t="s">
         <v>47</v>
@@ -23901,7 +23901,7 @@
         <v>34</v>
       </c>
       <c r="E383" t="s">
-        <v>818</v>
+        <v>819</v>
       </c>
       <c r="F383" t="s">
         <v>211</v>
@@ -23910,7 +23910,7 @@
         <v>41</v>
       </c>
       <c r="H383" t="s">
-        <v>819</v>
+        <v>425</v>
       </c>
       <c r="I383" t="s">
         <v>820</v>
@@ -23975,7 +23975,7 @@
         <v>320</v>
       </c>
       <c r="K384" t="s">
-        <v>122</v>
+        <v>75</v>
       </c>
       <c r="L384" t="s">
         <v>825</v>
@@ -24028,10 +24028,10 @@
         <v>828</v>
       </c>
       <c r="J385" t="s">
-        <v>320</v>
+        <v>58</v>
       </c>
       <c r="K385" t="s">
-        <v>96</v>
+        <v>202</v>
       </c>
       <c r="L385" t="s">
         <v>829</v>
@@ -24140,7 +24140,7 @@
         <v>835</v>
       </c>
       <c r="J387" t="s">
-        <v>685</v>
+        <v>681</v>
       </c>
       <c r="K387" t="s">
         <v>45</v>
@@ -24349,28 +24349,28 @@
         <v>33</v>
       </c>
       <c r="E391" t="s">
-        <v>672</v>
+        <v>851</v>
       </c>
       <c r="F391" t="s">
-        <v>40</v>
+        <v>211</v>
       </c>
       <c r="G391" t="s">
         <v>41</v>
       </c>
       <c r="H391" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="I391" t="s">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="J391" t="s">
-        <v>293</v>
+        <v>320</v>
       </c>
       <c r="K391" t="s">
-        <v>45</v>
+        <v>122</v>
       </c>
       <c r="L391" t="s">
-        <v>853</v>
+        <v>34</v>
       </c>
       <c r="M391" t="s">
         <v>850</v>
@@ -24382,7 +24382,7 @@
         <v>48</v>
       </c>
       <c r="P391" t="s">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="Q391" t="s">
         <v>47</v>
@@ -24405,28 +24405,28 @@
         <v>34</v>
       </c>
       <c r="E392" t="s">
+        <v>672</v>
+      </c>
+      <c r="F392" t="s">
+        <v>40</v>
+      </c>
+      <c r="G392" t="s">
+        <v>41</v>
+      </c>
+      <c r="H392" t="s">
         <v>854</v>
       </c>
-      <c r="F392" t="s">
-        <v>211</v>
-      </c>
-      <c r="G392" t="s">
-        <v>41</v>
-      </c>
-      <c r="H392" t="s">
+      <c r="I392" t="s">
         <v>855</v>
       </c>
-      <c r="I392" t="s">
+      <c r="J392" t="s">
+        <v>293</v>
+      </c>
+      <c r="K392" t="s">
+        <v>45</v>
+      </c>
+      <c r="L392" t="s">
         <v>856</v>
-      </c>
-      <c r="J392" t="s">
-        <v>320</v>
-      </c>
-      <c r="K392" t="s">
-        <v>122</v>
-      </c>
-      <c r="L392" t="s">
-        <v>34</v>
       </c>
       <c r="M392" t="s">
         <v>850</v>
@@ -24438,7 +24438,7 @@
         <v>48</v>
       </c>
       <c r="P392" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="Q392" t="s">
         <v>47</v>
@@ -24517,7 +24517,7 @@
         <v>34</v>
       </c>
       <c r="E394" t="s">
-        <v>672</v>
+        <v>861</v>
       </c>
       <c r="F394" t="s">
         <v>40</v>
@@ -24529,16 +24529,16 @@
         <v>846</v>
       </c>
       <c r="I394" t="s">
-        <v>861</v>
+        <v>862</v>
       </c>
       <c r="J394" t="s">
-        <v>293</v>
+        <v>101</v>
       </c>
       <c r="K394" t="s">
-        <v>859</v>
+        <v>45</v>
       </c>
       <c r="L394" t="s">
-        <v>862</v>
+        <v>863</v>
       </c>
       <c r="M394" t="s">
         <v>850</v>
@@ -24550,7 +24550,7 @@
         <v>48</v>
       </c>
       <c r="P394" t="s">
-        <v>861</v>
+        <v>862</v>
       </c>
       <c r="Q394" t="s">
         <v>47</v>
@@ -24573,7 +24573,7 @@
         <v>34</v>
       </c>
       <c r="E395" t="s">
-        <v>863</v>
+        <v>672</v>
       </c>
       <c r="F395" t="s">
         <v>40</v>
@@ -24588,10 +24588,10 @@
         <v>864</v>
       </c>
       <c r="J395" t="s">
-        <v>101</v>
+        <v>293</v>
       </c>
       <c r="K395" t="s">
-        <v>45</v>
+        <v>859</v>
       </c>
       <c r="L395" t="s">
         <v>865</v>
@@ -24812,7 +24812,7 @@
         <v>878</v>
       </c>
       <c r="J399" t="s">
-        <v>685</v>
+        <v>681</v>
       </c>
       <c r="K399" t="s">
         <v>45</v>
@@ -24865,7 +24865,7 @@
         <v>877</v>
       </c>
       <c r="I400" t="s">
-        <v>808</v>
+        <v>820</v>
       </c>
       <c r="J400" t="s">
         <v>58</v>
@@ -24886,7 +24886,7 @@
         <v>48</v>
       </c>
       <c r="P400" t="s">
-        <v>808</v>
+        <v>820</v>
       </c>
       <c r="Q400" t="s">
         <v>47</v>
@@ -25077,7 +25077,7 @@
         <v>33</v>
       </c>
       <c r="E404" t="s">
-        <v>763</v>
+        <v>672</v>
       </c>
       <c r="F404" t="s">
         <v>40</v>
@@ -25092,10 +25092,10 @@
         <v>898</v>
       </c>
       <c r="J404" t="s">
-        <v>178</v>
+        <v>681</v>
       </c>
       <c r="K404" t="s">
-        <v>178</v>
+        <v>45</v>
       </c>
       <c r="L404" t="s">
         <v>899</v>
@@ -25133,7 +25133,7 @@
         <v>34</v>
       </c>
       <c r="E405" t="s">
-        <v>672</v>
+        <v>763</v>
       </c>
       <c r="F405" t="s">
         <v>40</v>
@@ -25148,10 +25148,10 @@
         <v>901</v>
       </c>
       <c r="J405" t="s">
-        <v>685</v>
+        <v>178</v>
       </c>
       <c r="K405" t="s">
-        <v>45</v>
+        <v>178</v>
       </c>
       <c r="L405" t="s">
         <v>902</v>

</xml_diff>